<commit_message>
Dodatek roczny: korekta nieobecności oceniana w obie strony, zabezpieczenie przy braku rekordu korekty
Pierwotna nieobecność (Korygowana == true) pomijana tylko, gdy widoczny
jest rekord KorektaNieobecności; w przeciwnym razie oceniana jak dotąd.
Nowy scenariusz TS-21: L4 skorygowane na urlop na żądanie -> 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FM4CsinshuFUKmUUCkYkha
</commit_message>
<xml_diff>
--- a/ElementyPlac/Dodatek roczny - scenariusze testowe.xlsx
+++ b/ElementyPlac/Dodatek roczny - scenariusze testowe.xlsx
@@ -1763,8 +1763,68 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="K22" s="6" t="n"/>
+    <row r="22" ht="135" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TS-21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Bramka 3 – korekta nieobecności</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>L4 skorygowane na urlop na żądanie</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Jak TS-01, plus zwolnienie chorobowe (L4) w 2026 rozliczone na wypłacie, a następnie skorygowane (korekta nieobecności) na „Urlop wypoczynkowy” z przyczyną „Na żądanie”. Obie nieobecności łamią frekwencję.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>0. Przygotuj pracownika jak TS-01, dodaj „Zwolnienie chorobowe” w 2026 i rozlicz je na wypłacie.
+0a. Wykonaj korektę tej nieobecności na „Urlop wypoczynkowy”, Przyczyna = Na żądanie.
+1. Kartoteka pracownika → Etat → Dodatki: „Dodatek roczny”, Okres 1.01.2026–31.12.2026, Podstawa 1500,00 PLN.
+2. Płace → Listy płac: lista LPE za 01/2027 z tym pracownikiem → przelicz.
+3. Wypłata → element „Dodatek roczny” → kwota i zakładka „Zapis obliczeń”.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Dodatek = 0,00 PLN (korekta zamienia L4 na urlop na żądanie, który też łamie frekwencję).</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>…
+  - pominięta (skorygowana): Zwolnienie chorobowe (&lt;okres&gt;)
+  - łamiąca frekwencję: Urlop wypoczynkowy (&lt;okres&gt;)
+- frekwencja 100% w całym okresie: False
+…
+=&gt; wynik: 0,00</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>brak – do przygotowania</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Nieprzeprowadzony</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="n"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Kierunek odwrotny do TS-20: korekta z łamiącej na łamiącą. Jeśli w zapisie jest „UWAGA … brak rekordu korekty”, enova nie pokazuje korekty jako osobnego wiersza — wynik nadal 0, ale zgłosić.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="K23" s="6" t="n"/>

</xml_diff>